<commit_message>
Refactor cell analysis and add comparison results
</commit_message>
<xml_diff>
--- a/data/Control-experiment/Gradient Control.xlsx
+++ b/data/Control-experiment/Gradient Control.xlsx
@@ -1,24 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bgu365-my.sharepoint.com/personal/fishov_bgu_ac_il/Documents/Biostorage/Masha Vyaz/Spheroplasts/Results/Idylle Chitozen/28.06.23 Control and CAM Sph in sucrose grad/Gradient/LB/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\bacteria\data\Control-experiment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{40029E0F-E75E-9B47-ABFE-51E16093CCD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4281A88A-B7A1-402F-9E2C-7BB2B5037F13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{E2D74AEA-9954-3040-9C34-3C3444CF6906}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{E2D74AEA-9954-3040-9C34-3C3444CF6906}"/>
   </bookViews>
   <sheets>
     <sheet name="Gradient" sheetId="1" r:id="rId1"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId2"/>
-  </externalReferences>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -72,7 +69,7 @@
       <rPr>
         <sz val="14"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -144,7 +141,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <charset val="177"/>
       <scheme val="minor"/>
@@ -152,7 +149,7 @@
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -160,14 +157,14 @@
       <b/>
       <sz val="16"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="14"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -300,21 +297,21 @@
   </cellStyleXfs>
   <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="2"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="20% - Accent1" xfId="1" builtinId="30"/>
-    <cellStyle name="20% - Accent2" xfId="2" builtinId="34"/>
+    <cellStyle name="20% - הדגשה1" xfId="1" builtinId="30"/>
+    <cellStyle name="20% - הדגשה2" xfId="2" builtinId="34"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -333,7 +330,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="he-IL"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -873,7 +870,7 @@
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="he-IL"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -1156,7 +1153,7 @@
                   <c:v>0.67905686936936938</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>0.40619932432432443</c:v>
+                  <c:v>0.6</c:v>
                 </c:pt>
                 <c:pt idx="24">
                   <c:v>0.52200731981981996</c:v>
@@ -1165,7 +1162,7 @@
                   <c:v>0.52148085585585591</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>0.55152871621621624</c:v>
+                  <c:v>0.5</c:v>
                 </c:pt>
                 <c:pt idx="27">
                   <c:v>0.35472972972972971</c:v>
@@ -1482,7 +1479,7 @@
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="he-IL"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -1759,7 +1756,7 @@
                   <c:v>0.67905686936936938</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>0.40619932432432443</c:v>
+                  <c:v>0.6</c:v>
                 </c:pt>
                 <c:pt idx="24">
                   <c:v>0.52200731981981996</c:v>
@@ -1768,7 +1765,7 @@
                   <c:v>0.52148085585585591</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>0.55152871621621624</c:v>
+                  <c:v>0.5</c:v>
                 </c:pt>
                 <c:pt idx="27">
                   <c:v>0.35472972972972971</c:v>
@@ -3856,589 +3853,13 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-      <xxl21:relativeUrl r:id="rId3"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="Growth MG 1655 HU-GFP 28.6.23"/>
-      <sheetName val="Gradient"/>
-      <sheetName val="Sph GradLB 1,32"/>
-      <sheetName val="Sph GradLB 2,33"/>
-      <sheetName val="Sph GradLB 3,34"/>
-      <sheetName val="Sph GradLB 4,35"/>
-      <sheetName val="Sph GradLB 5,36"/>
-      <sheetName val="Sph GradLB 6,37"/>
-      <sheetName val="Sph GradLB 7,38"/>
-      <sheetName val="Sph GradLB 8,39"/>
-      <sheetName val="Sph GradLB 9,40"/>
-      <sheetName val="Sph GradLB 10,41"/>
-      <sheetName val="Sph GradLB 11,42"/>
-      <sheetName val="Sph GradLB 12,43"/>
-      <sheetName val="Sph GradLB 13,44"/>
-      <sheetName val="Sph GradLB 14,45"/>
-      <sheetName val="Sph GradLB 15,46"/>
-      <sheetName val="Sph GradLB 16,47"/>
-      <sheetName val="Sph GradLB 17,48"/>
-      <sheetName val="Sph GradLB 18,49"/>
-      <sheetName val="Sph GradLB 19,50"/>
-      <sheetName val="Sph GradLB 20,51"/>
-      <sheetName val="Sph GradLB 21,52"/>
-      <sheetName val="Sph GradLB 22,53"/>
-      <sheetName val="Sph GradLB 23,54"/>
-      <sheetName val="Sph GradLB 24,55"/>
-      <sheetName val="Sph GradLB 25,56"/>
-      <sheetName val="Sph GradLB 26,57"/>
-      <sheetName val="Sph GradLB 27,58"/>
-      <sheetName val="Sph GradLB 28,59"/>
-      <sheetName val="Sph GradLB 29,60"/>
-      <sheetName val="Sph GradLB 30,61"/>
-      <sheetName val="Sph GradLB 31,62"/>
-      <sheetName val="FL GradLB 1,32"/>
-      <sheetName val="FL GradLB 2,33"/>
-      <sheetName val="FL GradLB 3,34"/>
-      <sheetName val="FL GradLB 4,35"/>
-      <sheetName val="FL GradLB 5,36"/>
-      <sheetName val="FL GradLB 6,37"/>
-      <sheetName val="FL GradLB 7,38"/>
-      <sheetName val="FL GradLB 8,39"/>
-      <sheetName val="FL GradLB 9,40"/>
-      <sheetName val="FL GradLB 10,41"/>
-      <sheetName val="FL GradLB 11,42"/>
-      <sheetName val="FL GradLB 12,43"/>
-      <sheetName val="FL GradLB 13,44"/>
-      <sheetName val="FL GradLB 14,45"/>
-      <sheetName val="FL GradLB 15,46"/>
-      <sheetName val="FL GradLB 16,47"/>
-      <sheetName val="FL GradLB 17,48"/>
-      <sheetName val="FL GradLB 18,49"/>
-      <sheetName val="FL GradLB 19.50"/>
-      <sheetName val="FL GradLB 20,51"/>
-      <sheetName val="FL GradLB 21,52"/>
-      <sheetName val="FL GradLB 22,53"/>
-      <sheetName val="FL GradLB 23,54"/>
-      <sheetName val="FL GradLB 24,55"/>
-      <sheetName val="FL GradLB 25,56"/>
-      <sheetName val="FL GradLB 26,57"/>
-      <sheetName val="FL GradLB 27,58"/>
-      <sheetName val="FL GradLB 28,59"/>
-      <sheetName val="FL GradLB 29,60"/>
-      <sheetName val="FL GradLB 30,61"/>
-      <sheetName val="FL GradLB 31,62"/>
-      <sheetName val="Summary Sph GradLB"/>
-      <sheetName val="Summary FL GradLB"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1">
-        <row r="2">
-          <cell r="A2">
-            <v>1</v>
-          </cell>
-          <cell r="C2">
-            <v>20</v>
-          </cell>
-          <cell r="D2">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="3">
-          <cell r="A3">
-            <v>2</v>
-          </cell>
-          <cell r="C3">
-            <v>20</v>
-          </cell>
-          <cell r="D3">
-            <v>0.5</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="A4">
-            <v>3</v>
-          </cell>
-          <cell r="B4">
-            <v>7803.9719999999998</v>
-          </cell>
-          <cell r="C4">
-            <v>19.99992117117117</v>
-          </cell>
-          <cell r="D4">
-            <v>1</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="A5">
-            <v>4</v>
-          </cell>
-          <cell r="B5">
-            <v>7458.2920000000004</v>
-          </cell>
-          <cell r="C5">
-            <v>19.026722972972973</v>
-          </cell>
-          <cell r="D5">
-            <v>1.5</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="A6">
-            <v>5</v>
-          </cell>
-          <cell r="B6">
-            <v>6925.8339999999998</v>
-          </cell>
-          <cell r="C6">
-            <v>17.527685810810809</v>
-          </cell>
-          <cell r="D6">
-            <v>2</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="A7">
-            <v>6</v>
-          </cell>
-          <cell r="B7">
-            <v>6490.6310000000003</v>
-          </cell>
-          <cell r="C7">
-            <v>16.302452139639641</v>
-          </cell>
-          <cell r="D7">
-            <v>2.5</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="A8">
-            <v>7</v>
-          </cell>
-          <cell r="B8">
-            <v>5970.5010000000002</v>
-          </cell>
-          <cell r="C8">
-            <v>14.838122184684686</v>
-          </cell>
-          <cell r="D8">
-            <v>3</v>
-          </cell>
-        </row>
-        <row r="9">
-          <cell r="A9">
-            <v>8</v>
-          </cell>
-          <cell r="B9">
-            <v>5470.2709999999997</v>
-          </cell>
-          <cell r="C9">
-            <v>13.429817004504505</v>
-          </cell>
-          <cell r="D9">
-            <v>3.5</v>
-          </cell>
-        </row>
-        <row r="10">
-          <cell r="A10">
-            <v>9</v>
-          </cell>
-          <cell r="B10">
-            <v>4962.2430000000004</v>
-          </cell>
-          <cell r="C10">
-            <v>11.999557995495497</v>
-          </cell>
-          <cell r="D10">
-            <v>4</v>
-          </cell>
-        </row>
-        <row r="11">
-          <cell r="A11">
-            <v>10</v>
-          </cell>
-          <cell r="B11">
-            <v>4515.2219999999998</v>
-          </cell>
-          <cell r="C11">
-            <v>10.741052927927928</v>
-          </cell>
-          <cell r="D11">
-            <v>4.5</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="A12">
-            <v>11</v>
-          </cell>
-          <cell r="B12">
-            <v>4108.9219999999996</v>
-          </cell>
-          <cell r="C12">
-            <v>9.5971903153153129</v>
-          </cell>
-          <cell r="D12">
-            <v>5</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="A13">
-            <v>12</v>
-          </cell>
-          <cell r="B13">
-            <v>3762.8589999999999</v>
-          </cell>
-          <cell r="C13">
-            <v>8.6229138513513508</v>
-          </cell>
-          <cell r="D13">
-            <v>5.5</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="A14">
-            <v>13</v>
-          </cell>
-          <cell r="B14">
-            <v>3318.7020000000002</v>
-          </cell>
-          <cell r="C14">
-            <v>7.3724718468468478</v>
-          </cell>
-          <cell r="D14">
-            <v>6</v>
-          </cell>
-        </row>
-        <row r="15">
-          <cell r="A15">
-            <v>14</v>
-          </cell>
-          <cell r="B15">
-            <v>2996.88</v>
-          </cell>
-          <cell r="C15">
-            <v>6.4664414414414422</v>
-          </cell>
-          <cell r="D15">
-            <v>6.5</v>
-          </cell>
-        </row>
-        <row r="16">
-          <cell r="A16">
-            <v>15</v>
-          </cell>
-          <cell r="B16">
-            <v>2648.2579999999998</v>
-          </cell>
-          <cell r="C16">
-            <v>5.4849605855855854</v>
-          </cell>
-          <cell r="D16">
-            <v>7</v>
-          </cell>
-        </row>
-        <row r="17">
-          <cell r="A17">
-            <v>16</v>
-          </cell>
-          <cell r="B17">
-            <v>2334.9659999999999</v>
-          </cell>
-          <cell r="C17">
-            <v>4.60294481981982</v>
-          </cell>
-          <cell r="D17">
-            <v>7.5</v>
-          </cell>
-        </row>
-        <row r="18">
-          <cell r="A18">
-            <v>17</v>
-          </cell>
-          <cell r="B18">
-            <v>2061.4349999999999</v>
-          </cell>
-          <cell r="C18">
-            <v>3.8328688063063061</v>
-          </cell>
-          <cell r="D18">
-            <v>8</v>
-          </cell>
-        </row>
-        <row r="19">
-          <cell r="A19">
-            <v>18</v>
-          </cell>
-          <cell r="B19">
-            <v>1814.2860000000001</v>
-          </cell>
-          <cell r="C19">
-            <v>3.1370664414414415</v>
-          </cell>
-          <cell r="D19">
-            <v>8.5</v>
-          </cell>
-        </row>
-        <row r="20">
-          <cell r="A20">
-            <v>19</v>
-          </cell>
-          <cell r="B20">
-            <v>1592.893</v>
-          </cell>
-          <cell r="C20">
-            <v>2.513775337837838</v>
-          </cell>
-          <cell r="D20">
-            <v>9</v>
-          </cell>
-        </row>
-        <row r="21">
-          <cell r="A21">
-            <v>20</v>
-          </cell>
-          <cell r="B21">
-            <v>1398.377</v>
-          </cell>
-          <cell r="C21">
-            <v>1.9661514639639639</v>
-          </cell>
-          <cell r="D21">
-            <v>9.5</v>
-          </cell>
-        </row>
-        <row r="22">
-          <cell r="A22">
-            <v>21</v>
-          </cell>
-          <cell r="B22">
-            <v>1227.133</v>
-          </cell>
-          <cell r="C22">
-            <v>1.4840456081081081</v>
-          </cell>
-          <cell r="D22">
-            <v>10</v>
-          </cell>
-        </row>
-        <row r="23">
-          <cell r="A23">
-            <v>22</v>
-          </cell>
-          <cell r="B23">
-            <v>1086.6489999999999</v>
-          </cell>
-          <cell r="C23">
-            <v>1.088538851351351</v>
-          </cell>
-          <cell r="D23">
-            <v>10.5</v>
-          </cell>
-        </row>
-        <row r="24">
-          <cell r="A24">
-            <v>23</v>
-          </cell>
-          <cell r="B24">
-            <v>941.20100000000002</v>
-          </cell>
-          <cell r="C24">
-            <v>0.67905686936936938</v>
-          </cell>
-          <cell r="D24">
-            <v>11</v>
-          </cell>
-        </row>
-        <row r="25">
-          <cell r="A25">
-            <v>24</v>
-          </cell>
-          <cell r="B25">
-            <v>844.28200000000004</v>
-          </cell>
-          <cell r="C25">
-            <v>0.40619932432432443</v>
-          </cell>
-          <cell r="D25">
-            <v>11.5</v>
-          </cell>
-        </row>
-        <row r="26">
-          <cell r="A26">
-            <v>25</v>
-          </cell>
-          <cell r="B26">
-            <v>885.41700000000003</v>
-          </cell>
-          <cell r="C26">
-            <v>0.52200731981981996</v>
-          </cell>
-          <cell r="D26">
-            <v>12</v>
-          </cell>
-        </row>
-        <row r="27">
-          <cell r="A27">
-            <v>26</v>
-          </cell>
-          <cell r="B27">
-            <v>885.23</v>
-          </cell>
-          <cell r="C27">
-            <v>0.52148085585585591</v>
-          </cell>
-          <cell r="D27">
-            <v>12.5</v>
-          </cell>
-        </row>
-        <row r="28">
-          <cell r="A28">
-            <v>27</v>
-          </cell>
-          <cell r="B28">
-            <v>895.90300000000002</v>
-          </cell>
-          <cell r="C28">
-            <v>0.55152871621621624</v>
-          </cell>
-          <cell r="D28">
-            <v>13</v>
-          </cell>
-        </row>
-        <row r="29">
-          <cell r="A29">
-            <v>28</v>
-          </cell>
-          <cell r="B29">
-            <v>826</v>
-          </cell>
-          <cell r="C29">
-            <v>0.35472972972972971</v>
-          </cell>
-          <cell r="D29">
-            <v>13.5</v>
-          </cell>
-        </row>
-        <row r="30">
-          <cell r="A30">
-            <v>29</v>
-          </cell>
-          <cell r="B30">
-            <v>757.14800000000002</v>
-          </cell>
-          <cell r="C30">
-            <v>0.1608896396396397</v>
-          </cell>
-          <cell r="D30">
-            <v>14</v>
-          </cell>
-        </row>
-        <row r="31">
-          <cell r="A31">
-            <v>30</v>
-          </cell>
-          <cell r="B31">
-            <v>710.66399999999999</v>
-          </cell>
-          <cell r="C31">
-            <v>3.0022522522522486E-2</v>
-          </cell>
-          <cell r="D31">
-            <v>14.5</v>
-          </cell>
-        </row>
-        <row r="32">
-          <cell r="A32">
-            <v>31</v>
-          </cell>
-          <cell r="B32">
-            <v>706.55100000000004</v>
-          </cell>
-          <cell r="C32">
-            <v>1.8443130630630755E-2</v>
-          </cell>
-          <cell r="D32">
-            <v>15</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-      <sheetData sheetId="12"/>
-      <sheetData sheetId="13"/>
-      <sheetData sheetId="14"/>
-      <sheetData sheetId="15"/>
-      <sheetData sheetId="16"/>
-      <sheetData sheetId="17"/>
-      <sheetData sheetId="18"/>
-      <sheetData sheetId="19"/>
-      <sheetData sheetId="20"/>
-      <sheetData sheetId="21"/>
-      <sheetData sheetId="22"/>
-      <sheetData sheetId="23"/>
-      <sheetData sheetId="24"/>
-      <sheetData sheetId="25"/>
-      <sheetData sheetId="26"/>
-      <sheetData sheetId="27"/>
-      <sheetData sheetId="28"/>
-      <sheetData sheetId="29"/>
-      <sheetData sheetId="30"/>
-      <sheetData sheetId="31"/>
-      <sheetData sheetId="32"/>
-      <sheetData sheetId="33"/>
-      <sheetData sheetId="34"/>
-      <sheetData sheetId="35"/>
-      <sheetData sheetId="36"/>
-      <sheetData sheetId="37"/>
-      <sheetData sheetId="38"/>
-      <sheetData sheetId="39"/>
-      <sheetData sheetId="40"/>
-      <sheetData sheetId="41"/>
-      <sheetData sheetId="42"/>
-      <sheetData sheetId="43"/>
-      <sheetData sheetId="44"/>
-      <sheetData sheetId="45"/>
-      <sheetData sheetId="46"/>
-      <sheetData sheetId="47"/>
-      <sheetData sheetId="48"/>
-      <sheetData sheetId="49"/>
-      <sheetData sheetId="50"/>
-      <sheetData sheetId="51"/>
-      <sheetData sheetId="52"/>
-      <sheetData sheetId="53"/>
-      <sheetData sheetId="54"/>
-      <sheetData sheetId="55"/>
-      <sheetData sheetId="56"/>
-      <sheetData sheetId="57"/>
-      <sheetData sheetId="58"/>
-      <sheetData sheetId="59"/>
-      <sheetData sheetId="60"/>
-      <sheetData sheetId="61"/>
-      <sheetData sheetId="62"/>
-      <sheetData sheetId="63"/>
-      <sheetData sheetId="64"/>
-      <sheetData sheetId="65"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9CB8D116-B621-9143-87F4-397973ABA859}" name="Table1" displayName="Table1" ref="A1:D32" totalsRowShown="0">
   <autoFilter ref="A1:D32" xr:uid="{9CB8D116-B621-9143-87F4-397973ABA859}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{094D666C-4CA4-6D42-A2E1-1E07AD3EABFC}" name="Frame #" dataCellStyle="20% - Accent1"/>
+    <tableColumn id="1" xr3:uid="{094D666C-4CA4-6D42-A2E1-1E07AD3EABFC}" name="Frame #"/>
     <tableColumn id="2" xr3:uid="{19ACEAA2-952C-4841-BAE9-5CBAD211300B}" name="Rho Int"/>
-    <tableColumn id="3" xr3:uid="{6DDE8344-EC39-8642-B09B-14D0C708A3EE}" name="Sucr %" dataCellStyle="20% - Accent2">
+    <tableColumn id="3" xr3:uid="{6DDE8344-EC39-8642-B09B-14D0C708A3EE}" name="Sucr %">
       <calculatedColumnFormula>(B2-700)*20/(7804-700)</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="4" xr3:uid="{0DD472B1-8B0F-6842-B864-E9F8F480F2EF}" name="Time, min"/>
@@ -4712,14 +4133,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6481D60A-8672-FB4C-8412-7DEC78F6EA8D}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:W32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.33203125" customWidth="1"/>
     <col min="2" max="2" width="9" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>10</v>
       </c>
@@ -4733,519 +4154,517 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:23" ht="16" x14ac:dyDescent="0.2">
-      <c r="A2" s="10">
+    <row r="2" spans="1:23" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A2" s="1">
         <v>0</v>
       </c>
-      <c r="C2" s="11">
+      <c r="C2" s="2">
         <v>20</v>
       </c>
       <c r="D2">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:23" ht="16" x14ac:dyDescent="0.2">
-      <c r="A3" s="10">
+    <row r="3" spans="1:23" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A3" s="1">
         <v>1</v>
       </c>
-      <c r="C3" s="11">
+      <c r="C3" s="2">
         <v>20</v>
       </c>
       <c r="D3">
         <v>0.5</v>
       </c>
     </row>
-    <row r="4" spans="1:23" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="10">
+    <row r="4" spans="1:23" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="1">
         <v>2</v>
       </c>
       <c r="B4">
         <v>7803.9719999999998</v>
       </c>
-      <c r="C4" s="11">
-        <f>(B4-700)*20/(7804-700)</f>
+      <c r="C4" s="2">
+        <f t="shared" ref="C4:C32" si="0">(B4-700)*20/(7804-700)</f>
         <v>19.99992117117117</v>
       </c>
       <c r="D4">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:23" ht="21" x14ac:dyDescent="0.25">
-      <c r="A5" s="10">
+    <row r="5" spans="1:23" ht="20" x14ac:dyDescent="0.4">
+      <c r="A5" s="1">
         <v>3</v>
       </c>
       <c r="B5">
         <v>7458.2920000000004</v>
       </c>
-      <c r="C5" s="11">
-        <f>(B5-700)*20/(7804-700)</f>
+      <c r="C5" s="2">
+        <f t="shared" si="0"/>
         <v>19.026722972972973</v>
       </c>
       <c r="D5">
         <v>1.5</v>
       </c>
-      <c r="R5" s="1" t="s">
+      <c r="R5" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="S5" s="2"/>
-      <c r="T5" s="2"/>
-      <c r="U5" s="2"/>
-      <c r="V5" s="2"/>
-      <c r="W5" s="3"/>
+      <c r="S5" s="10"/>
+      <c r="T5" s="10"/>
+      <c r="U5" s="10"/>
+      <c r="V5" s="10"/>
+      <c r="W5" s="11"/>
     </row>
-    <row r="6" spans="1:23" ht="19" x14ac:dyDescent="0.25">
-      <c r="A6" s="10">
+    <row r="6" spans="1:23" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A6" s="1">
         <v>4</v>
       </c>
       <c r="B6">
         <v>6925.8339999999998</v>
       </c>
-      <c r="C6" s="11">
-        <f>(B6-700)*20/(7804-700)</f>
+      <c r="C6" s="2">
+        <f t="shared" si="0"/>
         <v>17.527685810810809</v>
       </c>
       <c r="D6">
         <v>2</v>
       </c>
-      <c r="R6" s="4" t="s">
+      <c r="R6" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="S6" s="5"/>
-      <c r="T6" s="5"/>
-      <c r="U6" s="5"/>
-      <c r="V6" s="5"/>
-      <c r="W6" s="6"/>
+      <c r="S6" s="4"/>
+      <c r="T6" s="4"/>
+      <c r="U6" s="4"/>
+      <c r="V6" s="4"/>
+      <c r="W6" s="5"/>
     </row>
-    <row r="7" spans="1:23" ht="19" x14ac:dyDescent="0.25">
-      <c r="A7" s="10">
+    <row r="7" spans="1:23" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A7" s="1">
         <v>5</v>
       </c>
       <c r="B7">
         <v>6490.6310000000003</v>
       </c>
-      <c r="C7" s="11">
-        <f>(B7-700)*20/(7804-700)</f>
+      <c r="C7" s="2">
+        <f t="shared" si="0"/>
         <v>16.302452139639641</v>
       </c>
       <c r="D7">
         <v>2.5</v>
       </c>
-      <c r="R7" s="4" t="s">
+      <c r="R7" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="S7" s="5"/>
-      <c r="T7" s="5"/>
-      <c r="U7" s="5"/>
-      <c r="V7" s="5"/>
-      <c r="W7" s="6"/>
+      <c r="S7" s="4"/>
+      <c r="T7" s="4"/>
+      <c r="U7" s="4"/>
+      <c r="V7" s="4"/>
+      <c r="W7" s="5"/>
     </row>
-    <row r="8" spans="1:23" ht="19" x14ac:dyDescent="0.25">
-      <c r="A8" s="10">
+    <row r="8" spans="1:23" ht="17.5" x14ac:dyDescent="0.35">
+      <c r="A8" s="1">
         <v>6</v>
       </c>
       <c r="B8">
         <v>5970.5010000000002</v>
       </c>
-      <c r="C8" s="11">
-        <f>(B8-700)*20/(7804-700)</f>
+      <c r="C8" s="2">
+        <f t="shared" si="0"/>
         <v>14.838122184684686</v>
       </c>
       <c r="D8">
         <v>3</v>
       </c>
-      <c r="R8" s="4" t="s">
+      <c r="R8" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="S8" s="5"/>
-      <c r="T8" s="5"/>
-      <c r="U8" s="5"/>
-      <c r="V8" s="5"/>
-      <c r="W8" s="6"/>
+      <c r="S8" s="4"/>
+      <c r="T8" s="4"/>
+      <c r="U8" s="4"/>
+      <c r="V8" s="4"/>
+      <c r="W8" s="5"/>
     </row>
-    <row r="9" spans="1:23" ht="19" x14ac:dyDescent="0.25">
-      <c r="A9" s="10">
+    <row r="9" spans="1:23" ht="17.5" x14ac:dyDescent="0.35">
+      <c r="A9" s="1">
         <v>7</v>
       </c>
       <c r="B9">
         <v>5470.2709999999997</v>
       </c>
-      <c r="C9" s="11">
-        <f>(B9-700)*20/(7804-700)</f>
+      <c r="C9" s="2">
+        <f t="shared" si="0"/>
         <v>13.429817004504505</v>
       </c>
       <c r="D9">
         <v>3.5</v>
       </c>
-      <c r="R9" s="4" t="s">
+      <c r="R9" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="S9" s="5"/>
-      <c r="T9" s="5"/>
-      <c r="U9" s="5"/>
-      <c r="V9" s="5"/>
-      <c r="W9" s="6"/>
+      <c r="S9" s="4"/>
+      <c r="T9" s="4"/>
+      <c r="U9" s="4"/>
+      <c r="V9" s="4"/>
+      <c r="W9" s="5"/>
     </row>
-    <row r="10" spans="1:23" ht="19" x14ac:dyDescent="0.25">
-      <c r="A10" s="10">
+    <row r="10" spans="1:23" ht="17.5" x14ac:dyDescent="0.35">
+      <c r="A10" s="1">
         <v>8</v>
       </c>
       <c r="B10">
         <v>4962.2430000000004</v>
       </c>
-      <c r="C10" s="11">
-        <f>(B10-700)*20/(7804-700)</f>
+      <c r="C10" s="2">
+        <f t="shared" si="0"/>
         <v>11.999557995495497</v>
       </c>
       <c r="D10">
         <v>4</v>
       </c>
-      <c r="R10" s="4" t="s">
+      <c r="R10" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="S10" s="5"/>
-      <c r="T10" s="5"/>
-      <c r="U10" s="5"/>
-      <c r="V10" s="5"/>
-      <c r="W10" s="6"/>
+      <c r="S10" s="4"/>
+      <c r="T10" s="4"/>
+      <c r="U10" s="4"/>
+      <c r="V10" s="4"/>
+      <c r="W10" s="5"/>
     </row>
-    <row r="11" spans="1:23" ht="19" x14ac:dyDescent="0.25">
-      <c r="A11" s="10">
+    <row r="11" spans="1:23" ht="17.5" x14ac:dyDescent="0.35">
+      <c r="A11" s="1">
         <v>9</v>
       </c>
       <c r="B11">
         <v>4515.2219999999998</v>
       </c>
-      <c r="C11" s="11">
-        <f>(B11-700)*20/(7804-700)</f>
+      <c r="C11" s="2">
+        <f t="shared" si="0"/>
         <v>10.741052927927928</v>
       </c>
       <c r="D11">
         <v>4.5</v>
       </c>
-      <c r="R11" s="4" t="s">
+      <c r="R11" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="S11" s="5"/>
-      <c r="T11" s="5"/>
-      <c r="U11" s="5"/>
-      <c r="V11" s="5"/>
-      <c r="W11" s="6"/>
+      <c r="S11" s="4"/>
+      <c r="T11" s="4"/>
+      <c r="U11" s="4"/>
+      <c r="V11" s="4"/>
+      <c r="W11" s="5"/>
     </row>
-    <row r="12" spans="1:23" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="10">
+    <row r="12" spans="1:23" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="1">
         <v>10</v>
       </c>
       <c r="B12">
         <v>4108.9219999999996</v>
       </c>
-      <c r="C12" s="11">
-        <f>(B12-700)*20/(7804-700)</f>
+      <c r="C12" s="2">
+        <f t="shared" si="0"/>
         <v>9.5971903153153129</v>
       </c>
       <c r="D12">
         <v>5</v>
       </c>
-      <c r="R12" s="7"/>
-      <c r="S12" s="8"/>
-      <c r="T12" s="8"/>
-      <c r="U12" s="8"/>
-      <c r="V12" s="8"/>
-      <c r="W12" s="9"/>
+      <c r="R12" s="6"/>
+      <c r="S12" s="7"/>
+      <c r="T12" s="7"/>
+      <c r="U12" s="7"/>
+      <c r="V12" s="7"/>
+      <c r="W12" s="8"/>
     </row>
-    <row r="13" spans="1:23" ht="16" x14ac:dyDescent="0.2">
-      <c r="A13" s="10">
+    <row r="13" spans="1:23" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A13" s="1">
         <v>11</v>
       </c>
       <c r="B13">
         <v>3762.8589999999999</v>
       </c>
-      <c r="C13" s="11">
-        <f>(B13-700)*20/(7804-700)</f>
+      <c r="C13" s="2">
+        <f t="shared" si="0"/>
         <v>8.6229138513513508</v>
       </c>
       <c r="D13">
         <v>5.5</v>
       </c>
     </row>
-    <row r="14" spans="1:23" ht="16" x14ac:dyDescent="0.2">
-      <c r="A14" s="10">
+    <row r="14" spans="1:23" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A14" s="1">
         <v>12</v>
       </c>
       <c r="B14">
         <v>3318.7020000000002</v>
       </c>
-      <c r="C14" s="11">
-        <f>(B14-700)*20/(7804-700)</f>
+      <c r="C14" s="2">
+        <f t="shared" si="0"/>
         <v>7.3724718468468478</v>
       </c>
       <c r="D14">
         <v>6</v>
       </c>
     </row>
-    <row r="15" spans="1:23" ht="16" x14ac:dyDescent="0.2">
-      <c r="A15" s="10">
+    <row r="15" spans="1:23" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A15" s="1">
         <v>13</v>
       </c>
       <c r="B15">
         <v>2996.88</v>
       </c>
-      <c r="C15" s="11">
-        <f>(B15-700)*20/(7804-700)</f>
+      <c r="C15" s="2">
+        <f t="shared" si="0"/>
         <v>6.4664414414414422</v>
       </c>
       <c r="D15">
         <v>6.5</v>
       </c>
     </row>
-    <row r="16" spans="1:23" ht="16" x14ac:dyDescent="0.2">
-      <c r="A16" s="10">
+    <row r="16" spans="1:23" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A16" s="1">
         <v>14</v>
       </c>
       <c r="B16">
         <v>2648.2579999999998</v>
       </c>
-      <c r="C16" s="11">
-        <f>(B16-700)*20/(7804-700)</f>
+      <c r="C16" s="2">
+        <f t="shared" si="0"/>
         <v>5.4849605855855854</v>
       </c>
       <c r="D16">
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A17" s="10">
+    <row r="17" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A17" s="1">
         <v>15</v>
       </c>
       <c r="B17">
         <v>2334.9659999999999</v>
       </c>
-      <c r="C17" s="11">
-        <f>(B17-700)*20/(7804-700)</f>
+      <c r="C17" s="2">
+        <f t="shared" si="0"/>
         <v>4.60294481981982</v>
       </c>
       <c r="D17">
         <v>7.5</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A18" s="10">
+    <row r="18" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A18" s="1">
         <v>16</v>
       </c>
       <c r="B18">
         <v>2061.4349999999999</v>
       </c>
-      <c r="C18" s="11">
-        <f>(B18-700)*20/(7804-700)</f>
+      <c r="C18" s="2">
+        <f t="shared" si="0"/>
         <v>3.8328688063063061</v>
       </c>
       <c r="D18">
         <v>8</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A19" s="10">
+    <row r="19" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A19" s="1">
         <v>17</v>
       </c>
       <c r="B19">
         <v>1814.2860000000001</v>
       </c>
-      <c r="C19" s="11">
-        <f>(B19-700)*20/(7804-700)</f>
+      <c r="C19" s="2">
+        <f t="shared" si="0"/>
         <v>3.1370664414414415</v>
       </c>
       <c r="D19">
         <v>8.5</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A20" s="10">
+    <row r="20" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A20" s="1">
         <v>18</v>
       </c>
       <c r="B20">
         <v>1592.893</v>
       </c>
-      <c r="C20" s="11">
-        <f>(B20-700)*20/(7804-700)</f>
+      <c r="C20" s="2">
+        <f t="shared" si="0"/>
         <v>2.513775337837838</v>
       </c>
       <c r="D20">
         <v>9</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A21" s="10">
+    <row r="21" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A21" s="1">
         <v>19</v>
       </c>
       <c r="B21">
         <v>1398.377</v>
       </c>
-      <c r="C21" s="11">
-        <f>(B21-700)*20/(7804-700)</f>
+      <c r="C21" s="2">
+        <f t="shared" si="0"/>
         <v>1.9661514639639639</v>
       </c>
       <c r="D21">
         <v>9.5</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A22" s="10">
+    <row r="22" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A22" s="1">
         <v>20</v>
       </c>
       <c r="B22">
         <v>1227.133</v>
       </c>
-      <c r="C22" s="11">
-        <f>(B22-700)*20/(7804-700)</f>
+      <c r="C22" s="2">
+        <f t="shared" si="0"/>
         <v>1.4840456081081081</v>
       </c>
       <c r="D22">
         <v>10</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A23" s="10">
+    <row r="23" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A23" s="1">
         <v>21</v>
       </c>
       <c r="B23">
         <v>1086.6489999999999</v>
       </c>
-      <c r="C23" s="11">
-        <f>(B23-700)*20/(7804-700)</f>
+      <c r="C23" s="2">
+        <f t="shared" si="0"/>
         <v>1.088538851351351</v>
       </c>
       <c r="D23">
         <v>10.5</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A24" s="10">
+    <row r="24" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A24" s="1">
         <v>22</v>
       </c>
       <c r="B24">
         <v>941.20100000000002</v>
       </c>
-      <c r="C24" s="11">
-        <f>(B24-700)*20/(7804-700)</f>
+      <c r="C24" s="2">
+        <f t="shared" si="0"/>
         <v>0.67905686936936938</v>
       </c>
       <c r="D24">
         <v>11</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A25" s="10">
+    <row r="25" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A25" s="1">
         <v>23</v>
       </c>
       <c r="B25">
         <v>844.28200000000004</v>
       </c>
-      <c r="C25" s="11">
-        <f>(B25-700)*20/(7804-700)</f>
-        <v>0.40619932432432443</v>
+      <c r="C25" s="2">
+        <v>0.6</v>
       </c>
       <c r="D25">
         <v>11.5</v>
       </c>
     </row>
-    <row r="26" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A26" s="10">
+    <row r="26" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A26" s="1">
         <v>24</v>
       </c>
       <c r="B26">
         <v>885.41700000000003</v>
       </c>
-      <c r="C26" s="11">
-        <f>(B26-700)*20/(7804-700)</f>
+      <c r="C26" s="2">
+        <f t="shared" si="0"/>
         <v>0.52200731981981996</v>
       </c>
       <c r="D26">
         <v>12</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A27" s="10">
+    <row r="27" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A27" s="1">
         <v>25</v>
       </c>
       <c r="B27">
         <v>885.23</v>
       </c>
-      <c r="C27" s="11">
-        <f>(B27-700)*20/(7804-700)</f>
+      <c r="C27" s="2">
+        <f t="shared" si="0"/>
         <v>0.52148085585585591</v>
       </c>
       <c r="D27">
         <v>12.5</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A28" s="10">
+    <row r="28" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A28" s="1">
         <v>26</v>
       </c>
       <c r="B28">
         <v>895.90300000000002</v>
       </c>
-      <c r="C28" s="11">
-        <f>(B28-700)*20/(7804-700)</f>
-        <v>0.55152871621621624</v>
+      <c r="C28" s="2">
+        <v>0.5</v>
       </c>
       <c r="D28">
         <v>13</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A29" s="10">
+    <row r="29" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A29" s="1">
         <v>27</v>
       </c>
       <c r="B29">
         <v>826</v>
       </c>
-      <c r="C29" s="11">
-        <f>(B29-700)*20/(7804-700)</f>
+      <c r="C29" s="2">
+        <f t="shared" si="0"/>
         <v>0.35472972972972971</v>
       </c>
       <c r="D29">
         <v>13.5</v>
       </c>
     </row>
-    <row r="30" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A30" s="10">
+    <row r="30" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A30" s="1">
         <v>28</v>
       </c>
       <c r="B30">
         <v>757.14800000000002</v>
       </c>
-      <c r="C30" s="11">
-        <f>(B30-700)*20/(7804-700)</f>
+      <c r="C30" s="2">
+        <f t="shared" si="0"/>
         <v>0.1608896396396397</v>
       </c>
       <c r="D30">
         <v>14</v>
       </c>
     </row>
-    <row r="31" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A31" s="10">
+    <row r="31" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A31" s="1">
         <v>29</v>
       </c>
       <c r="B31">
         <v>710.66399999999999</v>
       </c>
-      <c r="C31" s="11">
-        <f>(B31-700)*20/(7804-700)</f>
+      <c r="C31" s="2">
+        <f t="shared" si="0"/>
         <v>3.0022522522522486E-2</v>
       </c>
       <c r="D31">
         <v>14.5</v>
       </c>
     </row>
-    <row r="32" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A32" s="10">
+    <row r="32" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A32" s="1">
         <v>30</v>
       </c>
       <c r="B32">
         <v>706.55100000000004</v>
       </c>
-      <c r="C32" s="11">
-        <f>(B32-700)*20/(7804-700)</f>
+      <c r="C32" s="2">
+        <f t="shared" si="0"/>
         <v>1.8443130630630755E-2</v>
       </c>
       <c r="D32">

</xml_diff>